<commit_message>
Update report: 해안면 20260316_20260317
</commit_message>
<xml_diff>
--- a/shucle_report/해안면/20260316_20260317/report_해안면_20260316_20260317.xlsx
+++ b/shucle_report/해안면/20260316_20260317/report_해안면_20260316_20260317.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1차 핵심지표" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2차 세부지표_변동" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2차 세부지표_안정" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="핵심 해석" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="핵심 해석" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="부록_2차 세부지표_안정" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>분석기간: 2026.03.16 ~ 03.17 | 비교기간: 2026.03.12 ~ 03.13 | 생성: 2026-03-18 16:56 | 차트: 95개</t>
+          <t>분석기간: 2026.03.16 ~ 03.17 | 비교기간: 2026.03.12 ~ 03.13 | 생성: 2026-03-18 17:15 | 차트: 95개</t>
         </is>
       </c>
     </row>
@@ -582,12 +582,12 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>4.00건</t>
+          <t>4.0건</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>7.50건</t>
+          <t>7.5건</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -619,12 +619,12 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>4.00건</t>
+          <t>4.0건</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>6.50건</t>
+          <t>6.5건</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -656,12 +656,12 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>4.50명</t>
+          <t>4.5명</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>6.50명</t>
+          <t>6.5명</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>4.50명</t>
+          <t>4.5명</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>4.31분</t>
+          <t>4.3분</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>3.65분</t>
+          <t>3.6분</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -767,12 +767,12 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>0.81배</t>
+          <t>0.8배</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>1.25배</t>
+          <t>1.3배</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -804,12 +804,12 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>3.92분</t>
+          <t>3.9분</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>4.50분</t>
+          <t>4.5분</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -841,12 +841,12 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>1.00대</t>
+          <t>1.0대</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>1.00대</t>
+          <t>1.0대</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -878,12 +878,12 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>7.03시간</t>
+          <t>7.0시간</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>7.01시간</t>
+          <t>7.0시간</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1026,12 +1026,12 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>2.50명</t>
+          <t>2.5명</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>5.50명</t>
+          <t>5.5명</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -1063,12 +1063,12 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>2.00명</t>
+          <t>2.0명</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>2.50명</t>
+          <t>2.5명</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -1180,17 +1180,17 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>4.00</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>6.50</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>+2.50</t>
+          <t>+2.5</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -1217,17 +1217,17 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>4.31</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>3.65</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>-0.66</t>
+          <t>-0.7</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -1409,17 +1409,17 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1446,17 +1446,17 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -1483,17 +1483,17 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>+1.00</t>
+          <t>+1.0</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1564,17 +1564,17 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>6.50</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>+2.00</t>
+          <t>+2.0</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -1756,17 +1756,17 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>+0.93</t>
+          <t>+0.9</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
@@ -1793,17 +1793,17 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>3.92</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>+0.58</t>
+          <t>+0.6</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -1830,17 +1830,17 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>6.50</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>+2.00</t>
+          <t>+2.0</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
@@ -1911,17 +1911,17 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>+0.10</t>
+          <t>+0.1</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -1985,17 +1985,17 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>+0.45</t>
+          <t>+0.4</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
@@ -2177,17 +2177,17 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>6.50</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>+4.00</t>
+          <t>+4.0</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
@@ -2214,17 +2214,17 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>4.00</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>+7.00</t>
+          <t>+7.0</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
@@ -2369,17 +2369,17 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>4.00</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>7.50</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>+3.50</t>
+          <t>+3.5</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
@@ -2406,17 +2406,17 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>5.00</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -2524,17 +2524,17 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>+0.50</t>
+          <t>+0.5</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>+4.00</t>
+          <t>+4.0</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2598,17 +2598,17 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.1</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
@@ -2635,17 +2635,17 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>4.31</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>3.65</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>-0.66</t>
+          <t>-0.7</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>9.00</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>+5.00</t>
+          <t>+5.0</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
@@ -2753,17 +2753,17 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>5.50</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>+3.00</t>
+          <t>+3.0</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr">
@@ -2800,6 +2800,75 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>3. 핵심 해석</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>• 수요 증가: 호출(+88%), 이동완료(+62%), 탑승객(+44%) 모두 상승 — 분석기간 운행 2일(03/16,03/17), 비교기간 2일</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>• 이동완료율 100.0% → 86.7% (-13.3%p): 호출 8건 중 6건 완료 (호출취소 0건, 배차실패 2건)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>• 대기시간 개선: 4.3분 → 3.6분 (-15%) — 특히 03/17 상위10% 대기시간 9.5분으로 극단치 발생</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>• 가호출 성공률 급락: 90.0% → 79.5%, 가호출 시도 일평균 11.0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>• 성장 지표 긍정적: DAU +120%, 신규회원 2→2명(+25%), 누적 15명 — 이용자 기반 확대 추세</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>• 이동시간 증가: 3.9분 → 4.5분 (+15%) — 우회비율은 소폭 증가, 경로 효율성 저하</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2815,7 +2884,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>3. 2차 세부지표_안정 (10% 이내 변동)</t>
+          <t>4. [부록] 2차 세부지표_안정 (10% 이내 변동)</t>
         </is>
       </c>
     </row>
@@ -2876,17 +2945,17 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>4.31</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>3.65</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>-0.66</t>
+          <t>-0.7</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -2950,17 +3019,17 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>8.90</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>8.40</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-0.50</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -3024,17 +3093,17 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -3061,17 +3130,17 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>4.00</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>7.50</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>+3.50</t>
+          <t>+3.5</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -3142,17 +3211,17 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -3179,17 +3248,17 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -3216,17 +3285,17 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>+1.00</t>
+          <t>+1.0</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -3297,17 +3366,17 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>7.05</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>7.05</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
@@ -3334,17 +3403,17 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>9.05</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>9.05</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>+0.00</t>
+          <t>+0.0</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -3371,7 +3440,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -3404,59 +3473,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>4. 핵심 해석</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>• 대기시간 개선: 4.31분 → 3.65분 (-15%) — 특히 03/17 상위10% 대기시간 9.5분으로 극단치 발생</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>• 가호출 성공률 급락: 90.0% → 79.5%, 가호출 시도 일평균 11.0건</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>• 성장 지표 긍정적: DAU +120%, 누적 15명</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>• 이동시간 증가: 3.92분 → 4.50분 (+15%) — 우회비율은 소폭 증가, 경로 효율성 저하</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>